<commit_message>
He escogido el modelo de crecimiento y estoy escogiendo los vasos que han sido creados en cada fecha
</commit_message>
<xml_diff>
--- a/Datos_Modificados_Qca.xlsx
+++ b/Datos_Modificados_Qca.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\minicores\R_analisis\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\minicores\Qca_Bruto\Minicores-Q.canariensis\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FBFCC347-C061-4559-A5EC-B4648804A32C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4BEFE34B-7B97-41AB-8595-D74D67505789}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" firstSheet="2" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4410" yWindow="3630" windowWidth="21600" windowHeight="11295" tabRatio="500" firstSheet="12" activeTab="16" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="2Feb21" sheetId="1" r:id="rId1"/>
@@ -6347,7 +6347,7 @@
         <v>37</v>
       </c>
       <c r="K3">
-        <v>1.5271999999999999</v>
+        <v>1.6272</v>
       </c>
     </row>
     <row r="4" spans="1:18" x14ac:dyDescent="0.25">
@@ -6383,7 +6383,7 @@
         <v>37</v>
       </c>
       <c r="K4" s="88">
-        <v>1.8148</v>
+        <v>2</v>
       </c>
     </row>
     <row r="5" spans="1:18" x14ac:dyDescent="0.25">
@@ -6418,7 +6418,7 @@
         <v>37</v>
       </c>
       <c r="K5">
-        <v>0.55330000000000001</v>
+        <v>0.65329999999999999</v>
       </c>
     </row>
     <row r="6" spans="1:18" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -6453,7 +6453,7 @@
         <v>37</v>
       </c>
       <c r="K6">
-        <v>0.83250000000000002</v>
+        <v>1.2</v>
       </c>
     </row>
     <row r="7" spans="1:18" x14ac:dyDescent="0.25">
@@ -6548,7 +6548,7 @@
         <v>37</v>
       </c>
       <c r="K9">
-        <v>1.7496</v>
+        <v>1.496</v>
       </c>
     </row>
     <row r="10" spans="1:18" x14ac:dyDescent="0.25">
@@ -6568,13 +6568,13 @@
         <v>29</v>
       </c>
       <c r="F10">
-        <v>1.2177</v>
+        <v>1</v>
       </c>
       <c r="G10">
-        <v>1.2379</v>
+        <v>1</v>
       </c>
       <c r="H10">
-        <v>1.1483000000000001</v>
+        <v>1</v>
       </c>
       <c r="I10" s="12">
         <v>1.25</v>
@@ -6645,7 +6645,7 @@
       <c r="I12" s="12"/>
       <c r="J12" s="12"/>
       <c r="K12" s="89">
-        <v>4.5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="13" spans="1:18" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
He actualizado el código, me queda pasarlo a limpio y añadir un par de modificaciones
</commit_message>
<xml_diff>
--- a/Datos_Modificados_Qca.xlsx
+++ b/Datos_Modificados_Qca.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\minicores\Qca_Bruto\Minicores-Q.canariensis\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4BEFE34B-7B97-41AB-8595-D74D67505789}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6D6F7C11-7EA0-4D57-8400-69FF8B76740E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4410" yWindow="3630" windowWidth="21600" windowHeight="11295" tabRatio="500" firstSheet="12" activeTab="16" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-705" windowWidth="29040" windowHeight="15720" tabRatio="500" firstSheet="9" activeTab="12" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="2Feb21" sheetId="1" r:id="rId1"/>
@@ -3623,19 +3623,19 @@
       </c>
       <c r="E7" s="80"/>
       <c r="F7">
-        <v>1.4475</v>
+        <v>1.2</v>
       </c>
       <c r="G7">
-        <v>1.4475</v>
+        <v>1.1719999999999999</v>
       </c>
       <c r="H7">
-        <v>1.4475</v>
+        <v>1.2250000000000001</v>
       </c>
       <c r="I7" s="81">
         <v>1.4</v>
       </c>
       <c r="J7" s="87">
-        <v>0.67030000000000001</v>
+        <v>0.84</v>
       </c>
     </row>
     <row r="8" spans="1:12" x14ac:dyDescent="0.25">
@@ -4343,7 +4343,7 @@
     <col min="1013" max="1021" width="9.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>3</v>
       </c>
@@ -4375,7 +4375,7 @@
         <v>197</v>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2" s="7">
         <v>2</v>
       </c>
@@ -4407,7 +4407,7 @@
         <v>1.2619</v>
       </c>
     </row>
-    <row r="3" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="7">
         <v>3</v>
       </c>
@@ -4439,7 +4439,7 @@
         <v>1.7709999999999999</v>
       </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4" s="7">
         <v>5</v>
       </c>
@@ -4465,7 +4465,7 @@
         <v>1.841</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5" s="7">
         <v>8</v>
       </c>
@@ -4497,7 +4497,7 @@
         <v>0.3745</v>
       </c>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A6" s="7">
         <v>9</v>
       </c>
@@ -4529,7 +4529,7 @@
         <v>0.87570000000000003</v>
       </c>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A7" s="7">
         <v>10</v>
       </c>
@@ -4561,7 +4561,7 @@
         <v>0.60209999999999997</v>
       </c>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A8" s="7">
         <v>18</v>
       </c>
@@ -4593,7 +4593,7 @@
         <v>1.956</v>
       </c>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A9" s="7">
         <v>19</v>
       </c>
@@ -4619,7 +4619,7 @@
         <v>1.2251000000000001</v>
       </c>
     </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A10" s="7">
         <v>26</v>
       </c>
@@ -4651,7 +4651,7 @@
         <v>0.74270000000000003</v>
       </c>
     </row>
-    <row r="11" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="7">
         <v>30</v>
       </c>
@@ -4680,7 +4680,7 @@
         <v>1.9516</v>
       </c>
     </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A12" s="7">
         <v>36</v>
       </c>
@@ -4712,7 +4712,7 @@
         <v>0.45369999999999999</v>
       </c>
     </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A13" s="7">
         <v>40</v>
       </c>
@@ -4744,7 +4744,7 @@
         <v>1.4204000000000001</v>
       </c>
     </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A14" s="7">
         <v>44</v>
       </c>
@@ -4760,17 +4760,21 @@
         <v>0.503</v>
       </c>
       <c r="G14">
-        <v>0.503</v>
+        <v>0.51919999999999999</v>
       </c>
       <c r="H14">
         <v>0.503</v>
       </c>
       <c r="I14" s="12"/>
       <c r="J14">
-        <v>0.98640000000000005</v>
-      </c>
-    </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
+        <v>0.71799999999999997</v>
+      </c>
+      <c r="K14">
+        <f>AVERAGE(F14:H14)/J14</f>
+        <v>0.70807799442896935</v>
+      </c>
+    </row>
+    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A15" s="7">
         <v>47</v>
       </c>
@@ -5339,6 +5343,7 @@
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="4" max="4" width="10" customWidth="1"/>
+    <col min="11" max="11" width="11.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:17" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -5489,7 +5494,7 @@
         <v>1.1156999999999999</v>
       </c>
       <c r="G5">
-        <v>1.0998000000000001</v>
+        <v>1.1021000000000001</v>
       </c>
       <c r="H5">
         <v>1.0919000000000001</v>
@@ -5498,7 +5503,7 @@
         <v>1.3</v>
       </c>
       <c r="J5">
-        <v>0.91569999999999996</v>
+        <v>0.86</v>
       </c>
     </row>
     <row r="6" spans="1:17" ht="23.25" x14ac:dyDescent="0.25">
@@ -5650,7 +5655,7 @@
       </c>
       <c r="I10" s="12"/>
       <c r="J10">
-        <v>0.61899999999999999</v>
+        <v>0.44</v>
       </c>
     </row>
     <row r="11" spans="1:17" ht="23.25" x14ac:dyDescent="0.25">
@@ -5919,19 +5924,19 @@
         <v>41</v>
       </c>
       <c r="F6">
-        <v>0.44579999999999997</v>
+        <v>0.5</v>
       </c>
       <c r="G6">
         <v>0.44579999999999997</v>
       </c>
       <c r="H6">
-        <v>0.42309999999999998</v>
+        <v>0.56999999999999995</v>
       </c>
       <c r="I6" s="12">
         <v>0.46</v>
       </c>
       <c r="J6">
-        <v>0.60489999999999999</v>
+        <v>0.56000000000000005</v>
       </c>
     </row>
     <row r="7" spans="1:12" ht="23.25" x14ac:dyDescent="0.25">
@@ -11750,7 +11755,7 @@
         <v>37</v>
       </c>
       <c r="L7" s="87">
-        <v>0.67030000000000001</v>
+        <v>0.8</v>
       </c>
     </row>
     <row r="8" spans="1:12" x14ac:dyDescent="0.25">

</xml_diff>